<commit_message>
Replace the saved latest packages with the 55p ones; read the SE netting claim off the sheet
examples/{bst,se,taxi,ltd}-latest are the populated 2026-27 packages from
this run, the copy the generate workflows make. categoryNetting takes the
mileage claim from the year-end Purchases tab so a corrupted Admin rate trips
only its own checks. The judge indicator tests follow the regenerated reports.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Model: claude-sonnet-5-5
Claude-Session: https://claude.ai/code/session_01VyobNtzoueeNnQKC2bkP4e
</commit_message>
<xml_diff>
--- a/examples/ltd-latest/expensesform.xlsx
+++ b/examples/ltd-latest/expensesform.xlsx
@@ -1748,10 +1748,10 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -3154,11 +3154,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 09'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -4561,11 +4561,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 10'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -5968,11 +5968,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 11'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -7378,11 +7378,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 01'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -8785,11 +8785,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 02'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -10192,11 +10192,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 03'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -11599,11 +11599,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 04'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -13006,11 +13006,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 05'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -14413,11 +14413,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 06'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -15820,11 +15820,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 07'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>
@@ -17227,11 +17227,11 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="19" t="str">
         <f aca="false">"Mileage Claim @ "&amp;TEXT(C30*100,0)&amp;"p"</f>
-        <v>Mileage Claim @ 45p</v>
+        <v>Mileage Claim @ 55p</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">'Month 08'!C30</f>
-        <v>0.45</v>
+        <v>0.55</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">SUM(D10:D29)</f>

</xml_diff>